<commit_message>
Fixed the bug modifier key input after long press.
</commit_message>
<xml_diff>
--- a/keymap.xlsx
+++ b/keymap.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1215" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1221" uniqueCount="189">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -3171,8 +3171,12 @@
         <v>1</v>
       </c>
       <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
+      <c r="H22" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>1</v>
+      </c>
       <c r="J22" s="6"/>
       <c r="K22" s="2" t="s">
         <v>44</v>
@@ -3403,8 +3407,12 @@
         <v>49</v>
       </c>
       <c r="G30" s="8"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="3"/>
+      <c r="H30" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>1</v>
+      </c>
       <c r="J30" s="6"/>
       <c r="K30" s="2" t="s">
         <v>44</v>
@@ -3880,8 +3888,12 @@
         <v>19</v>
       </c>
       <c r="G46" s="3"/>
-      <c r="H46" s="2"/>
-      <c r="I46" s="3"/>
+      <c r="H46" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I46" s="3" t="s">
+        <v>1</v>
+      </c>
       <c r="J46" s="6"/>
       <c r="K46" s="2" t="s">
         <v>44</v>

</xml_diff>

<commit_message>
Fixed the issue key mouse does not work.
</commit_message>
<xml_diff>
--- a/keymap.xlsx
+++ b/keymap.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="space modifier" sheetId="1" state="visible" r:id="rId2"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="161">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -426,58 +426,67 @@
     <t xml:space="preserve">F13修飾</t>
   </si>
   <si>
+    <t xml:space="preserve">Reload</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Space修飾</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ひらがな./変換/無変換　修飾</t>
+  </si>
+  <si>
+    <t xml:space="preserve">!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&amp;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(</t>
+  </si>
+  <si>
+    <t xml:space="preserve">)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">?</t>
+  </si>
+  <si>
     <t xml:space="preserve">_</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Space修飾</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ひらがな./変換/無変換　修飾</t>
-  </si>
-  <si>
-    <t xml:space="preserve">!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">“</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$</t>
-  </si>
-  <si>
-    <t xml:space="preserve">%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&amp;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(</t>
-  </si>
-  <si>
-    <t xml:space="preserve">)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">?</t>
   </si>
   <si>
     <t xml:space="preserve">セミコロン　修飾</t>
@@ -2751,23 +2760,15 @@
       <c r="O17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2"/>
+      <c r="A18" s="3" t="s">
+        <v>134</v>
+      </c>
       <c r="B18" s="3"/>
-      <c r="C18" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>66</v>
-      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="3"/>
       <c r="J18" s="2"/>
@@ -2811,9 +2812,7 @@
       <c r="K19" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L19" s="2" t="s">
-        <v>81</v>
-      </c>
+      <c r="L19" s="2"/>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -2853,7 +2852,9 @@
         <v>19</v>
       </c>
       <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
+      <c r="M20" s="2" t="s">
+        <v>135</v>
+      </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
     </row>
@@ -2880,18 +2881,12 @@
         <v>92</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>94</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="I21" s="3"/>
+      <c r="J21" s="2"/>
       <c r="K21" s="2"/>
-      <c r="L21" s="2" t="s">
-        <v>134</v>
-      </c>
+      <c r="L21" s="2"/>
       <c r="M21" s="2" t="s">
         <v>33</v>
       </c>
@@ -2974,7 +2969,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B25" s="16"/>
       <c r="C25" s="11"/>
@@ -2997,21 +2992,11 @@
     <row r="26" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
-      <c r="C26" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>66</v>
-      </c>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="3"/>
       <c r="J26" s="2"/>
@@ -3053,9 +3038,7 @@
       <c r="K27" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L27" s="2" t="s">
-        <v>81</v>
-      </c>
+      <c r="L27" s="2"/>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -3093,7 +3076,9 @@
         <v>19</v>
       </c>
       <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
+      <c r="M28" s="2" t="s">
+        <v>135</v>
+      </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
     </row>
@@ -3120,18 +3105,12 @@
         <v>92</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="I29" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>94</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="I29" s="3"/>
+      <c r="J29" s="2"/>
       <c r="K29" s="2"/>
-      <c r="L29" s="2" t="s">
-        <v>134</v>
-      </c>
+      <c r="L29" s="2"/>
       <c r="M29" s="2" t="s">
         <v>33</v>
       </c>
@@ -3207,7 +3186,7 @@
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="11"/>
@@ -3309,37 +3288,37 @@
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3"/>
       <c r="B36" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="L36" s="10" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="M36" s="10" t="s">
         <v>94</v>
@@ -3385,7 +3364,7 @@
         <v>33</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>18</v>
@@ -3406,16 +3385,16 @@
         <v>2</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>134</v>
+        <v>154</v>
       </c>
       <c r="M37" s="2" t="s">
         <v>33</v>
@@ -3526,7 +3505,7 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="11"/>
@@ -3546,21 +3525,11 @@
     <row r="42" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
-      <c r="C42" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D42" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>66</v>
-      </c>
+      <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
       <c r="H42" s="2"/>
       <c r="I42" s="3"/>
       <c r="J42" s="2"/>
@@ -3602,9 +3571,7 @@
       <c r="K43" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L43" s="2" t="s">
-        <v>81</v>
-      </c>
+      <c r="L43" s="2"/>
       <c r="M43" s="2"/>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -3642,7 +3609,9 @@
         <v>30</v>
       </c>
       <c r="L44" s="2"/>
-      <c r="M44" s="2"/>
+      <c r="M44" s="2" t="s">
+        <v>135</v>
+      </c>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
     </row>
@@ -3669,14 +3638,10 @@
         <v>92</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="I45" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="J45" s="2" t="s">
-        <v>94</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="I45" s="3"/>
+      <c r="J45" s="2"/>
       <c r="K45" s="2"/>
       <c r="L45" s="2"/>
       <c r="M45" s="2" t="s">
@@ -3754,7 +3719,7 @@
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="16" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B49" s="16"/>
       <c r="C49" s="11"/>
@@ -3815,14 +3780,14 @@
       <c r="E52" s="4"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="I52" s="3"/>
       <c r="J52" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="K52" s="2"/>
       <c r="L52" s="2"/>
@@ -3838,7 +3803,7 @@
       <c r="E53" s="2"/>
       <c r="F53" s="3"/>
       <c r="G53" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="H53" s="2"/>
       <c r="I53" s="3"/>
@@ -4709,7 +4674,7 @@
       </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2" t="s">
-        <v>134</v>
+        <v>154</v>
       </c>
       <c r="M21" s="2" t="s">
         <v>33</v>
@@ -4793,7 +4758,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B25" s="16"/>
       <c r="C25" s="11"/>
@@ -4949,7 +4914,7 @@
       </c>
       <c r="K29" s="2"/>
       <c r="L29" s="2" t="s">
-        <v>134</v>
+        <v>154</v>
       </c>
       <c r="M29" s="2" t="s">
         <v>33</v>
@@ -5026,7 +4991,7 @@
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="11"/>
@@ -5128,37 +5093,37 @@
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3"/>
       <c r="B36" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="L36" s="10" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="M36" s="10" t="s">
         <v>94</v>
@@ -5204,7 +5169,7 @@
         <v>33</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>18</v>
@@ -5225,16 +5190,16 @@
         <v>2</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>134</v>
+        <v>154</v>
       </c>
       <c r="M37" s="2" t="s">
         <v>33</v>
@@ -5345,7 +5310,7 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="11"/>
@@ -5573,7 +5538,7 @@
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="16" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B49" s="16"/>
       <c r="C49" s="11"/>
@@ -5634,14 +5599,14 @@
       <c r="E52" s="4"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="I52" s="3"/>
       <c r="J52" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="K52" s="2"/>
       <c r="L52" s="2"/>
@@ -5657,7 +5622,7 @@
       <c r="E53" s="2"/>
       <c r="F53" s="3"/>
       <c r="G53" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="H53" s="2"/>
       <c r="I53" s="3"/>

</xml_diff>

<commit_message>
Updated new key bind.
</commit_message>
<xml_diff>
--- a/keymap.xlsx
+++ b/keymap.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="966" uniqueCount="162">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -429,15 +429,36 @@
     <t xml:space="preserve">Reload</t>
   </si>
   <si>
+    <t xml:space="preserve">C+;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+-</t>
+  </si>
+  <si>
     <t xml:space="preserve">C+]</t>
   </si>
   <si>
-    <t xml:space="preserve">C+-</t>
-  </si>
-  <si>
     <t xml:space="preserve">Space修飾</t>
   </si>
   <si>
+    <t xml:space="preserve">セミコロン　修飾</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Space+ F13 修飾</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+Home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+←</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+→</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C+End</t>
+  </si>
+  <si>
     <t xml:space="preserve">ひらがな./変換/無変換　修飾</t>
   </si>
   <si>
@@ -487,24 +508,6 @@
   </si>
   <si>
     <t xml:space="preserve">_</t>
-  </si>
-  <si>
-    <t xml:space="preserve">セミコロン　修飾</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Space+ F13 修飾</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+Home</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+←</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+→</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+End</t>
   </si>
 </sst>
 </file>
@@ -719,7 +722,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -790,6 +793,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -2184,7 +2191,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AA55"/>
+  <dimension ref="A1:AA62"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="1" style="1" width="7.66"/>
@@ -2812,7 +2819,9 @@
       <c r="K19" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L19" s="2"/>
+      <c r="L19" s="2" t="s">
+        <v>135</v>
+      </c>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -2851,9 +2860,11 @@
       <c r="K20" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="L20" s="2"/>
+      <c r="L20" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="M20" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -2880,8 +2891,8 @@
       <c r="G21" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="H21" s="2" t="s">
-        <v>136</v>
+      <c r="H21" s="3" t="s">
+        <v>54</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="2"/>
@@ -2969,7 +2980,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B25" s="16"/>
       <c r="C25" s="11"/>
@@ -3038,7 +3049,9 @@
       <c r="K27" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="L27" s="2"/>
+      <c r="L27" s="2" t="s">
+        <v>135</v>
+      </c>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -3075,9 +3088,11 @@
       <c r="K28" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="L28" s="2"/>
+      <c r="L28" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="M28" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -3104,8 +3119,8 @@
       <c r="G29" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="H29" s="2" t="s">
-        <v>136</v>
+      <c r="H29" s="3" t="s">
+        <v>54</v>
       </c>
       <c r="I29" s="3"/>
       <c r="J29" s="2"/>
@@ -3186,7 +3201,7 @@
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="11"/>
@@ -3205,123 +3220,97 @@
     </row>
     <row r="34" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3"/>
-      <c r="B34" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="I34" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="J34" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="L34" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="M34" s="2" t="s">
-        <v>72</v>
-      </c>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
+      <c r="L34" s="2"/>
+      <c r="M34" s="2"/>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="3"/>
       <c r="B35" s="3" t="s">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>98</v>
+        <v>75</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>100</v>
+        <v>76</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>77</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>103</v>
+        <v>5</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>104</v>
+        <v>52</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>105</v>
+        <v>79</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="L35" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="M35" s="10" t="s">
-        <v>108</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="L35" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="M35" s="2"/>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3"/>
       <c r="B36" s="3" t="s">
-        <v>139</v>
+        <v>82</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>140</v>
+        <v>83</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>141</v>
+        <v>84</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>142</v>
+        <v>85</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>143</v>
+        <v>86</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>144</v>
+        <v>87</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>145</v>
+        <v>53</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>146</v>
+        <v>54</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="L36" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="M36" s="10" t="s">
-        <v>94</v>
+        <v>55</v>
+      </c>
+      <c r="K36" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>137</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -3364,38 +3353,30 @@
         <v>33</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>150</v>
+        <v>88</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>18</v>
+        <v>89</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>91</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="G37" s="3" t="s">
-        <v>81</v>
+        <v>88</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>92</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="I37" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="J37" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="K37" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="L37" s="3" t="s">
-        <v>154</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="I37" s="3"/>
+      <c r="J37" s="2"/>
+      <c r="K37" s="2"/>
+      <c r="L37" s="2"/>
       <c r="M37" s="2" t="s">
         <v>33</v>
       </c>
@@ -3448,18 +3429,16 @@
       <c r="D38" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E38" s="8" t="s">
-        <v>48</v>
-      </c>
+      <c r="E38" s="3"/>
       <c r="F38" s="3" t="s">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="G38" s="3"/>
-      <c r="H38" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="I38" s="17" t="s">
-        <v>58</v>
+      <c r="H38" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>1</v>
       </c>
       <c r="J38" s="6"/>
       <c r="K38" s="2" t="s">
@@ -3475,11 +3454,11 @@
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
       <c r="G39" s="3"/>
-      <c r="H39" s="17"/>
-      <c r="I39" s="17"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="3"/>
       <c r="J39" s="6"/>
       <c r="K39" s="2"/>
       <c r="L39" s="2"/>
@@ -3504,8 +3483,8 @@
       <c r="O40" s="14"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7" t="s">
-        <v>155</v>
+      <c r="A41" s="16" t="s">
+        <v>140</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="11"/>
@@ -3541,143 +3520,79 @@
     </row>
     <row r="43" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="3"/>
-      <c r="B43" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G43" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="H43" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I43" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="J43" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="K43" s="2" t="s">
-        <v>80</v>
-      </c>
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="2"/>
+      <c r="K43" s="2"/>
       <c r="L43" s="2"/>
       <c r="M43" s="2"/>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="3"/>
-      <c r="B44" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>86</v>
-      </c>
+      <c r="A44" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="2"/>
       <c r="G44" s="2" t="s">
-        <v>87</v>
+        <v>141</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="I44" s="3" t="s">
-        <v>54</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="I44" s="3"/>
       <c r="J44" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="K44" s="8" t="s">
-        <v>30</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="K44" s="2"/>
       <c r="L44" s="2"/>
-      <c r="M44" s="2" t="s">
-        <v>135</v>
-      </c>
+      <c r="M44" s="2"/>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="F45" s="3" t="s">
-        <v>88</v>
-      </c>
+      <c r="A45" s="3"/>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="3"/>
       <c r="G45" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="H45" s="2" t="s">
-        <v>136</v>
-      </c>
+        <v>144</v>
+      </c>
+      <c r="H45" s="2"/>
       <c r="I45" s="3"/>
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
       <c r="L45" s="2"/>
-      <c r="M45" s="2" t="s">
-        <v>33</v>
-      </c>
+      <c r="M45" s="2"/>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>47</v>
-      </c>
+      <c r="A46" s="3"/>
+      <c r="B46" s="3"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
       <c r="E46" s="3"/>
-      <c r="F46" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G46" s="3"/>
-      <c r="H46" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="I46" s="3" t="s">
-        <v>1</v>
-      </c>
+      <c r="F46" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="G46" s="8"/>
+      <c r="H46" s="2"/>
+      <c r="I46" s="3"/>
       <c r="J46" s="6"/>
-      <c r="K46" s="2" t="s">
-        <v>44</v>
-      </c>
+      <c r="K46" s="2"/>
       <c r="L46" s="6"/>
       <c r="M46" s="2"/>
       <c r="N46" s="6"/>
@@ -3690,7 +3605,7 @@
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
+      <c r="G47" s="8"/>
       <c r="H47" s="2"/>
       <c r="I47" s="3"/>
       <c r="J47" s="6"/>
@@ -3718,8 +3633,8 @@
       <c r="O48" s="14"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="16" t="s">
-        <v>156</v>
+      <c r="A49" s="7" t="s">
+        <v>145</v>
       </c>
       <c r="B49" s="16"/>
       <c r="C49" s="11"/>
@@ -3738,96 +3653,200 @@
     </row>
     <row r="50" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="3"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
-      <c r="F50" s="2"/>
-      <c r="G50" s="2"/>
-      <c r="H50" s="2"/>
-      <c r="I50" s="3"/>
-      <c r="J50" s="2"/>
-      <c r="K50" s="2"/>
-      <c r="L50" s="2"/>
-      <c r="M50" s="2"/>
+      <c r="B50" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I50" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="K50" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="L50" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="M50" s="2" t="s">
+        <v>72</v>
+      </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
     </row>
     <row r="51" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="3"/>
-      <c r="B51" s="3"/>
-      <c r="C51" s="3"/>
-      <c r="D51" s="3"/>
-      <c r="E51" s="3"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="2"/>
-      <c r="H51" s="2"/>
-      <c r="I51" s="3"/>
-      <c r="J51" s="2"/>
-      <c r="K51" s="2"/>
-      <c r="L51" s="2"/>
-      <c r="M51" s="2"/>
+      <c r="B51" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="I51" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="L51" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="M51" s="10" t="s">
+        <v>108</v>
+      </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
     </row>
     <row r="52" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B52" s="3"/>
-      <c r="C52" s="3"/>
-      <c r="D52" s="3"/>
-      <c r="E52" s="4"/>
-      <c r="F52" s="2"/>
+      <c r="A52" s="3"/>
+      <c r="B52" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>150</v>
+      </c>
       <c r="G52" s="2" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="I52" s="3"/>
+        <v>152</v>
+      </c>
+      <c r="I52" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="J52" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="K52" s="2"/>
-      <c r="L52" s="2"/>
-      <c r="M52" s="2"/>
+        <v>154</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="L52" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="M52" s="10" t="s">
+        <v>94</v>
+      </c>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
     </row>
     <row r="53" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3"/>
-      <c r="B53" s="3"/>
-      <c r="C53" s="3"/>
-      <c r="D53" s="3"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="3"/>
-      <c r="G53" s="2" t="s">
+      <c r="A53" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="I53" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="J53" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="K53" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="H53" s="2"/>
-      <c r="I53" s="3"/>
-      <c r="J53" s="2"/>
-      <c r="K53" s="2"/>
-      <c r="L53" s="2"/>
-      <c r="M53" s="2"/>
+      <c r="L53" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="M53" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="3"/>
-      <c r="B54" s="3"/>
-      <c r="C54" s="3"/>
-      <c r="D54" s="3"/>
-      <c r="E54" s="3"/>
-      <c r="F54" s="8" t="s">
+      <c r="A54" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E54" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="F54" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="G54" s="8"/>
-      <c r="H54" s="2"/>
-      <c r="I54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="I54" s="17" t="s">
+        <v>58</v>
+      </c>
       <c r="J54" s="6"/>
-      <c r="K54" s="2"/>
+      <c r="K54" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="L54" s="6"/>
       <c r="M54" s="2"/>
       <c r="N54" s="6"/>
@@ -3838,17 +3857,143 @@
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
-      <c r="E55" s="3"/>
-      <c r="F55" s="3"/>
-      <c r="G55" s="8"/>
-      <c r="H55" s="2"/>
-      <c r="I55" s="3"/>
+      <c r="E55" s="8"/>
+      <c r="F55" s="8"/>
+      <c r="G55" s="3"/>
+      <c r="H55" s="17"/>
+      <c r="I55" s="17"/>
       <c r="J55" s="6"/>
       <c r="K55" s="2"/>
       <c r="L55" s="2"/>
       <c r="M55" s="2"/>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
+    </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="18"/>
+      <c r="B56" s="18"/>
+      <c r="C56" s="18"/>
+      <c r="D56" s="18"/>
+      <c r="E56" s="18"/>
+      <c r="F56" s="18"/>
+      <c r="G56" s="18"/>
+      <c r="H56" s="18"/>
+      <c r="I56" s="18"/>
+      <c r="J56" s="18"/>
+      <c r="K56" s="18"/>
+      <c r="L56" s="18"/>
+      <c r="M56" s="18"/>
+      <c r="N56" s="18"/>
+      <c r="O56" s="18"/>
+      <c r="P56" s="18"/>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="18"/>
+      <c r="B57" s="18"/>
+      <c r="C57" s="18"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="18"/>
+      <c r="F57" s="18"/>
+      <c r="G57" s="18"/>
+      <c r="H57" s="18"/>
+      <c r="I57" s="18"/>
+      <c r="J57" s="18"/>
+      <c r="K57" s="18"/>
+      <c r="L57" s="18"/>
+      <c r="M57" s="18"/>
+      <c r="N57" s="18"/>
+      <c r="O57" s="18"/>
+      <c r="P57" s="18"/>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="18"/>
+      <c r="B58" s="18"/>
+      <c r="C58" s="18"/>
+      <c r="D58" s="18"/>
+      <c r="E58" s="18"/>
+      <c r="F58" s="18"/>
+      <c r="G58" s="18"/>
+      <c r="H58" s="18"/>
+      <c r="I58" s="18"/>
+      <c r="J58" s="18"/>
+      <c r="K58" s="18"/>
+      <c r="L58" s="18"/>
+      <c r="M58" s="18"/>
+      <c r="N58" s="18"/>
+      <c r="O58" s="18"/>
+      <c r="P58" s="18"/>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="18"/>
+      <c r="B59" s="18"/>
+      <c r="C59" s="18"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
+      <c r="F59" s="18"/>
+      <c r="G59" s="18"/>
+      <c r="H59" s="18"/>
+      <c r="I59" s="18"/>
+      <c r="J59" s="18"/>
+      <c r="K59" s="18"/>
+      <c r="L59" s="18"/>
+      <c r="M59" s="18"/>
+      <c r="N59" s="18"/>
+      <c r="O59" s="18"/>
+      <c r="P59" s="18"/>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="18"/>
+      <c r="B60" s="18"/>
+      <c r="C60" s="18"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
+      <c r="F60" s="18"/>
+      <c r="G60" s="18"/>
+      <c r="H60" s="18"/>
+      <c r="I60" s="18"/>
+      <c r="J60" s="18"/>
+      <c r="K60" s="18"/>
+      <c r="L60" s="18"/>
+      <c r="M60" s="18"/>
+      <c r="N60" s="18"/>
+      <c r="O60" s="18"/>
+      <c r="P60" s="18"/>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="18"/>
+      <c r="B61" s="18"/>
+      <c r="C61" s="18"/>
+      <c r="D61" s="18"/>
+      <c r="E61" s="18"/>
+      <c r="F61" s="18"/>
+      <c r="G61" s="18"/>
+      <c r="H61" s="18"/>
+      <c r="I61" s="18"/>
+      <c r="J61" s="18"/>
+      <c r="K61" s="18"/>
+      <c r="L61" s="18"/>
+      <c r="M61" s="18"/>
+      <c r="N61" s="18"/>
+      <c r="O61" s="18"/>
+      <c r="P61" s="18"/>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="18"/>
+      <c r="B62" s="18"/>
+      <c r="C62" s="18"/>
+      <c r="D62" s="18"/>
+      <c r="E62" s="18"/>
+      <c r="F62" s="18"/>
+      <c r="G62" s="18"/>
+      <c r="H62" s="18"/>
+      <c r="I62" s="18"/>
+      <c r="J62" s="18"/>
+      <c r="K62" s="18"/>
+      <c r="L62" s="18"/>
+      <c r="M62" s="18"/>
+      <c r="N62" s="18"/>
+      <c r="O62" s="18"/>
+      <c r="P62" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="91">
@@ -4663,18 +4808,18 @@
       <c r="G21" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="H21" s="18" t="s">
+      <c r="H21" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="I21" s="18" t="s">
+      <c r="I21" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="J21" s="18" t="s">
+      <c r="J21" s="19" t="s">
         <v>94</v>
       </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="M21" s="2" t="s">
         <v>33</v>
@@ -4758,7 +4903,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B25" s="16"/>
       <c r="C25" s="11"/>
@@ -4822,13 +4967,13 @@
       <c r="F27" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G27" s="19" t="s">
+      <c r="G27" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="H27" s="19" t="s">
+      <c r="H27" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="I27" s="19" t="s">
+      <c r="I27" s="20" t="s">
         <v>52</v>
       </c>
       <c r="J27" s="2" t="s">
@@ -4846,34 +4991,34 @@
     </row>
     <row r="28" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3"/>
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="C28" s="19" t="s">
+      <c r="C28" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="D28" s="19" t="s">
+      <c r="D28" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="E28" s="19" t="s">
+      <c r="E28" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="F28" s="19" t="s">
+      <c r="F28" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="G28" s="19" t="s">
+      <c r="G28" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="H28" s="19" t="s">
+      <c r="H28" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="I28" s="19" t="s">
+      <c r="I28" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="J28" s="19" t="s">
+      <c r="J28" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="K28" s="19" t="s">
+      <c r="K28" s="20" t="s">
         <v>19</v>
       </c>
       <c r="L28" s="2"/>
@@ -4888,33 +5033,33 @@
       <c r="B29" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C29" s="19" t="s">
+      <c r="C29" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="D29" s="19" t="s">
+      <c r="D29" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="E29" s="19" t="s">
+      <c r="E29" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="F29" s="19" t="s">
+      <c r="F29" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="G29" s="19" t="s">
+      <c r="G29" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="H29" s="18" t="s">
+      <c r="H29" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="I29" s="18" t="s">
+      <c r="I29" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="J29" s="18" t="s">
+      <c r="J29" s="19" t="s">
         <v>94</v>
       </c>
       <c r="K29" s="2"/>
       <c r="L29" s="2" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="M29" s="2" t="s">
         <v>33</v>
@@ -4991,7 +5136,7 @@
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="11"/>
@@ -5093,37 +5238,37 @@
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3"/>
       <c r="B36" s="3" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="L36" s="10" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="M36" s="10" t="s">
         <v>94</v>
@@ -5169,7 +5314,7 @@
         <v>33</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>18</v>
@@ -5190,16 +5335,16 @@
         <v>2</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="M37" s="2" t="s">
         <v>33</v>
@@ -5310,7 +5455,7 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>155</v>
+        <v>139</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="11"/>
@@ -5538,7 +5683,7 @@
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="16" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="B49" s="16"/>
       <c r="C49" s="11"/>
@@ -5599,14 +5744,14 @@
       <c r="E52" s="4"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="I52" s="3"/>
       <c r="J52" s="2" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="K52" s="2"/>
       <c r="L52" s="2"/>
@@ -5622,7 +5767,7 @@
       <c r="E53" s="2"/>
       <c r="F53" s="3"/>
       <c r="G53" s="2" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="H53" s="2"/>
       <c r="I53" s="3"/>

</xml_diff>

<commit_message>
Updated F14 function to long_press_shift.ahk.
</commit_message>
<xml_diff>
--- a/keymap.xlsx
+++ b/keymap.xlsx
@@ -582,6 +582,9 @@
     <t xml:space="preserve">/ 修飾   C+k,C+{}</t>
   </si>
   <si>
+    <t xml:space="preserve">C+→</t>
+  </si>
+  <si>
     <t xml:space="preserve">C+q</t>
   </si>
   <si>
@@ -598,9 +601,6 @@
   </si>
   <si>
     <t xml:space="preserve">C+←</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C+→</t>
   </si>
   <si>
     <t xml:space="preserve">C+k</t>
@@ -678,7 +678,7 @@
       <charset val="128"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -711,26 +711,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFBBE33D"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFB2B2B2"/>
         <bgColor rgb="FFCCCCCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF81D41A"/>
-        <bgColor rgb="FFBBE33D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFBF00"/>
         <bgColor rgb="FFFF9900"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFBBE33D"/>
-        <bgColor rgb="FF81D41A"/>
       </patternFill>
     </fill>
   </fills>
@@ -845,7 +839,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -914,10 +908,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -926,15 +916,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -954,7 +944,7 @@
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFBBE33D"/>
+      <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
@@ -991,7 +981,7 @@
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF81D41A"/>
+      <rgbColor rgb="FFBBE33D"/>
       <rgbColor rgb="FFFFBF00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
@@ -3176,9 +3166,7 @@
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
-      <c r="Q13" s="3" t="s">
-        <v>33</v>
-      </c>
+      <c r="Q13" s="3"/>
       <c r="R13" s="3" t="s">
         <v>165</v>
       </c>
@@ -3212,9 +3200,7 @@
       <c r="AB13" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="AC13" s="2" t="s">
-        <v>33</v>
-      </c>
+      <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
       <c r="AE13" s="2"/>
     </row>
@@ -3254,35 +3240,17 @@
       </c>
       <c r="N14" s="6"/>
       <c r="O14" s="6"/>
-      <c r="Q14" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="R14" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="S14" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="T14" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="U14" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="V14" s="3" t="s">
-        <v>49</v>
-      </c>
+      <c r="Q14" s="3"/>
+      <c r="R14" s="3"/>
+      <c r="S14" s="3"/>
+      <c r="T14" s="3"/>
+      <c r="U14" s="3"/>
+      <c r="V14" s="3"/>
       <c r="W14" s="3"/>
-      <c r="X14" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="Y14" s="17" t="s">
-        <v>58</v>
-      </c>
+      <c r="X14" s="3"/>
+      <c r="Y14" s="3"/>
       <c r="Z14" s="6"/>
-      <c r="AA14" s="2" t="s">
-        <v>44</v>
-      </c>
+      <c r="AA14" s="2"/>
       <c r="AB14" s="6"/>
       <c r="AC14" s="2"/>
       <c r="AD14" s="6"/>
@@ -3314,11 +3282,11 @@
       <c r="R15" s="3"/>
       <c r="S15" s="3"/>
       <c r="T15" s="3"/>
-      <c r="U15" s="8"/>
-      <c r="V15" s="8"/>
+      <c r="U15" s="3"/>
+      <c r="V15" s="3"/>
       <c r="W15" s="3"/>
-      <c r="X15" s="17"/>
-      <c r="Y15" s="17"/>
+      <c r="X15" s="3"/>
+      <c r="Y15" s="3"/>
       <c r="Z15" s="6"/>
       <c r="AA15" s="2"/>
       <c r="AB15" s="2"/>
@@ -3364,7 +3332,7 @@
       <c r="Q17" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="R17" s="18"/>
+      <c r="R17" s="17"/>
       <c r="S17" s="12"/>
       <c r="T17" s="12"/>
       <c r="U17" s="12"/>
@@ -3492,9 +3460,11 @@
       <c r="J19" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="K19" s="2"/>
+      <c r="K19" s="3" t="s">
+        <v>54</v>
+      </c>
       <c r="L19" s="2" t="s">
-        <v>86</v>
+        <v>19</v>
       </c>
       <c r="M19" s="2" t="s">
         <v>79</v>
@@ -3573,7 +3543,9 @@
       <c r="K20" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="L20" s="2"/>
+      <c r="L20" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="M20" s="2" t="s">
         <v>80</v>
       </c>
@@ -3704,9 +3676,7 @@
       <c r="D22" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E22" s="3" t="s">
-        <v>1</v>
-      </c>
+      <c r="E22" s="3"/>
       <c r="F22" s="3" t="s">
         <v>49</v>
       </c>
@@ -3791,7 +3761,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7"/>
-      <c r="B24" s="19"/>
+      <c r="B24" s="18"/>
       <c r="C24" s="14"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
@@ -3810,7 +3780,7 @@
       <c r="A25" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="B25" s="18"/>
+      <c r="B25" s="17"/>
       <c r="C25" s="12"/>
       <c r="D25" s="12"/>
       <c r="E25" s="12"/>
@@ -3956,9 +3926,11 @@
       <c r="J27" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="K27" s="2"/>
+      <c r="K27" s="3" t="s">
+        <v>54</v>
+      </c>
       <c r="L27" s="2" t="s">
-        <v>86</v>
+        <v>19</v>
       </c>
       <c r="M27" s="2" t="s">
         <v>79</v>
@@ -4001,7 +3973,9 @@
       <c r="AB27" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="AC27" s="2"/>
+      <c r="AC27" s="2" t="s">
+        <v>79</v>
+      </c>
       <c r="AD27" s="2"/>
       <c r="AE27" s="2"/>
     </row>
@@ -4037,7 +4011,9 @@
       <c r="K28" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="L28" s="2"/>
+      <c r="L28" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="M28" s="2" t="s">
         <v>80</v>
       </c>
@@ -4080,7 +4056,7 @@
         <v>180</v>
       </c>
       <c r="AC28" s="2" t="s">
-        <v>181</v>
+        <v>80</v>
       </c>
       <c r="AD28" s="2"/>
       <c r="AE28" s="2"/>
@@ -4170,9 +4146,7 @@
       <c r="D30" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E30" s="3" t="s">
-        <v>1</v>
-      </c>
+      <c r="E30" s="3"/>
       <c r="F30" s="8" t="s">
         <v>49</v>
       </c>
@@ -4257,7 +4231,7 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7"/>
-      <c r="B32" s="19"/>
+      <c r="B32" s="18"/>
       <c r="C32" s="14"/>
       <c r="D32" s="14"/>
       <c r="E32" s="14"/>
@@ -4276,7 +4250,7 @@
       <c r="A33" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="B33" s="18"/>
+      <c r="B33" s="17"/>
       <c r="C33" s="12"/>
       <c r="D33" s="12"/>
       <c r="E33" s="12"/>
@@ -4293,7 +4267,7 @@
       <c r="Q33" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="R33" s="18"/>
+      <c r="R33" s="17"/>
       <c r="S33" s="12"/>
       <c r="T33" s="12"/>
       <c r="U33" s="12"/>
@@ -4348,7 +4322,9 @@
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
-      <c r="Q34" s="3"/>
+      <c r="Q34" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="R34" s="3" t="s">
         <v>109</v>
       </c>
@@ -4415,19 +4391,23 @@
         <v>52</v>
       </c>
       <c r="J35" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K35" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="L35" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="M35" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="K35" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="L35" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="M35" s="2"/>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
-      <c r="Q35" s="3"/>
-      <c r="R35" s="3" t="s">
+      <c r="Q35" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="R35" s="19" t="s">
         <v>74</v>
       </c>
       <c r="S35" s="3" t="s">
@@ -4442,25 +4422,27 @@
       <c r="V35" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="W35" s="20" t="s">
+      <c r="W35" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="X35" s="20" t="s">
+      <c r="X35" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="Y35" s="20" t="s">
+      <c r="Y35" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="Z35" s="2" t="s">
+      <c r="Z35" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA35" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB35" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="AC35" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="AA35" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="AB35" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="AC35" s="2"/>
       <c r="AD35" s="2"/>
       <c r="AE35" s="2"/>
     </row>
@@ -4493,22 +4475,24 @@
       <c r="J36" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="K36" s="8" t="s">
-        <v>30</v>
+      <c r="K36" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>180</v>
+        <v>86</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>181</v>
+        <v>80</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
-      <c r="Q36" s="3"/>
-      <c r="R36" s="3" t="s">
+      <c r="Q36" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="R36" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="S36" s="3" t="s">
+      <c r="S36" s="19" t="s">
         <v>83</v>
       </c>
       <c r="T36" s="3" t="s">
@@ -4517,29 +4501,29 @@
       <c r="U36" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="V36" s="20" t="s">
+      <c r="V36" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="W36" s="20" t="s">
+      <c r="W36" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="X36" s="20" t="s">
+      <c r="X36" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="Y36" s="20" t="s">
+      <c r="Y36" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z36" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="Z36" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="AA36" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB36" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="AC36" s="2" t="s">
-        <v>181</v>
+      <c r="AA36" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="AB36" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="AC36" s="19" t="s">
+        <v>80</v>
       </c>
       <c r="AD36" s="2"/>
       <c r="AE36" s="2"/>
@@ -4585,33 +4569,29 @@
       <c r="Q37" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="R37" s="20" t="s">
+      <c r="R37" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="S37" s="20" t="s">
+      <c r="S37" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="T37" s="20" t="s">
+      <c r="T37" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="U37" s="20" t="s">
+      <c r="U37" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="V37" s="20" t="s">
+      <c r="V37" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="W37" s="20" t="s">
+      <c r="W37" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="X37" s="20" t="s">
+      <c r="X37" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="Y37" s="20" t="s">
-        <v>180</v>
-      </c>
-      <c r="Z37" s="20" t="s">
-        <v>180</v>
-      </c>
+      <c r="Y37" s="3"/>
+      <c r="Z37" s="3"/>
       <c r="AA37" s="2"/>
       <c r="AB37" s="2"/>
       <c r="AC37" s="2" t="s">
@@ -4664,23 +4644,27 @@
       <c r="T38" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="U38" s="3"/>
+      <c r="U38" s="3" t="s">
+        <v>48</v>
+      </c>
       <c r="V38" s="3" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="W38" s="3"/>
-      <c r="X38" s="2" t="s">
-        <v>1</v>
+      <c r="X38" s="3" t="s">
+        <v>50</v>
       </c>
       <c r="Y38" s="3" t="s">
-        <v>1</v>
+        <v>58</v>
       </c>
       <c r="Z38" s="6"/>
       <c r="AA38" s="2" t="s">
         <v>44</v>
       </c>
       <c r="AB38" s="6"/>
-      <c r="AC38" s="2"/>
+      <c r="AC38" s="2" t="s">
+        <v>52</v>
+      </c>
       <c r="AD38" s="6"/>
       <c r="AE38" s="6"/>
     </row>
@@ -4707,17 +4691,23 @@
       <c r="U39" s="3"/>
       <c r="V39" s="3"/>
       <c r="W39" s="3"/>
-      <c r="X39" s="2"/>
+      <c r="X39" s="3"/>
       <c r="Y39" s="3"/>
       <c r="Z39" s="6"/>
       <c r="AA39" s="2"/>
-      <c r="AB39" s="2"/>
-      <c r="AC39" s="2"/>
-      <c r="AD39" s="2"/>
+      <c r="AB39" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC39" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD39" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="AE39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="19"/>
+      <c r="B40" s="18"/>
       <c r="C40" s="14"/>
       <c r="D40" s="14"/>
       <c r="E40" s="14"/>
@@ -4733,10 +4723,10 @@
       <c r="O40" s="15"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="18" t="s">
+      <c r="A41" s="17" t="s">
         <v>184</v>
       </c>
-      <c r="B41" s="18"/>
+      <c r="B41" s="17"/>
       <c r="C41" s="12"/>
       <c r="D41" s="12"/>
       <c r="E41" s="12"/>
@@ -4750,10 +4740,10 @@
       <c r="M41" s="12"/>
       <c r="N41" s="12"/>
       <c r="O41" s="13"/>
-      <c r="Q41" s="18" t="s">
+      <c r="Q41" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="R41" s="18"/>
+      <c r="R41" s="17"/>
       <c r="S41" s="12"/>
       <c r="T41" s="12"/>
       <c r="U41" s="12"/>
@@ -4810,7 +4800,9 @@
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
       <c r="I43" s="3"/>
-      <c r="J43" s="2"/>
+      <c r="J43" s="2" t="s">
+        <v>186</v>
+      </c>
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
       <c r="M43" s="2"/>
@@ -4818,7 +4810,7 @@
       <c r="O43" s="2"/>
       <c r="Q43" s="3"/>
       <c r="R43" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="S43" s="2"/>
       <c r="T43" s="2"/>
@@ -4826,14 +4818,14 @@
       <c r="V43" s="2"/>
       <c r="W43" s="2"/>
       <c r="X43" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="Y43" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="Z43" s="2"/>
       <c r="AA43" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="AB43" s="2"/>
       <c r="AC43" s="2"/>
@@ -4852,14 +4844,14 @@
       <c r="E44" s="4"/>
       <c r="F44" s="2"/>
       <c r="G44" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I44" s="3"/>
       <c r="J44" s="2" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
@@ -4871,9 +4863,7 @@
       <c r="S44" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="T44" s="2" t="s">
-        <v>23</v>
-      </c>
+      <c r="T44" s="2"/>
       <c r="U44" s="4" t="s">
         <v>85</v>
       </c>
@@ -4928,7 +4918,7 @@
       <c r="X45" s="3"/>
       <c r="Y45" s="3"/>
       <c r="Z45" s="2"/>
-      <c r="AA45" s="17" t="s">
+      <c r="AA45" s="20" t="s">
         <v>43</v>
       </c>
       <c r="AB45" s="2"/>
@@ -5021,8 +5011,8 @@
       <c r="AE47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="19"/>
-      <c r="B48" s="19"/>
+      <c r="A48" s="18"/>
+      <c r="B48" s="18"/>
       <c r="C48" s="14"/>
       <c r="D48" s="14"/>
       <c r="E48" s="14"/>
@@ -5041,7 +5031,7 @@
       <c r="A49" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="B49" s="18"/>
+      <c r="B49" s="17"/>
       <c r="C49" s="12"/>
       <c r="D49" s="12"/>
       <c r="E49" s="12"/>
@@ -5302,10 +5292,10 @@
         <v>49</v>
       </c>
       <c r="G54" s="3"/>
-      <c r="H54" s="17" t="s">
+      <c r="H54" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="I54" s="17" t="s">
+      <c r="I54" s="20" t="s">
         <v>58</v>
       </c>
       <c r="J54" s="6"/>
@@ -5323,8 +5313,8 @@
       <c r="U54" s="8"/>
       <c r="V54" s="3"/>
       <c r="W54" s="3"/>
-      <c r="X54" s="17"/>
-      <c r="Y54" s="17"/>
+      <c r="X54" s="20"/>
+      <c r="Y54" s="20"/>
       <c r="Z54" s="6"/>
       <c r="AA54" s="2"/>
       <c r="AB54" s="6"/>
@@ -5340,8 +5330,8 @@
       <c r="E55" s="8"/>
       <c r="F55" s="8"/>
       <c r="G55" s="3"/>
-      <c r="H55" s="17"/>
-      <c r="I55" s="17"/>
+      <c r="H55" s="20"/>
+      <c r="I55" s="20"/>
       <c r="J55" s="6"/>
       <c r="K55" s="2"/>
       <c r="L55" s="2"/>
@@ -5355,8 +5345,8 @@
       <c r="U55" s="8"/>
       <c r="V55" s="8"/>
       <c r="W55" s="3"/>
-      <c r="X55" s="17"/>
-      <c r="Y55" s="17"/>
+      <c r="X55" s="20"/>
+      <c r="Y55" s="20"/>
       <c r="Z55" s="6"/>
       <c r="AA55" s="2"/>
       <c r="AB55" s="2"/>
@@ -6472,7 +6462,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7"/>
-      <c r="B24" s="19"/>
+      <c r="B24" s="18"/>
       <c r="C24" s="14"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
@@ -6491,7 +6481,7 @@
       <c r="A25" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="B25" s="18"/>
+      <c r="B25" s="17"/>
       <c r="C25" s="12"/>
       <c r="D25" s="12"/>
       <c r="E25" s="12"/>
@@ -6553,13 +6543,13 @@
       <c r="F27" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G27" s="22" t="s">
+      <c r="G27" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="H27" s="22" t="s">
+      <c r="H27" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="I27" s="22" t="s">
+      <c r="I27" s="19" t="s">
         <v>52</v>
       </c>
       <c r="J27" s="2" t="s">
@@ -6577,34 +6567,34 @@
     </row>
     <row r="28" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3"/>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="D28" s="22" t="s">
+      <c r="D28" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="E28" s="22" t="s">
+      <c r="E28" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="F28" s="22" t="s">
+      <c r="F28" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="G28" s="22" t="s">
+      <c r="G28" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="H28" s="22" t="s">
+      <c r="H28" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="I28" s="22" t="s">
+      <c r="I28" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="J28" s="22" t="s">
+      <c r="J28" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="K28" s="22" t="s">
+      <c r="K28" s="19" t="s">
         <v>19</v>
       </c>
       <c r="L28" s="2"/>
@@ -6619,19 +6609,19 @@
       <c r="B29" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C29" s="22" t="s">
+      <c r="C29" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="D29" s="22" t="s">
+      <c r="D29" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="E29" s="22" t="s">
+      <c r="E29" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="F29" s="22" t="s">
+      <c r="F29" s="19" t="s">
         <v>88</v>
       </c>
-      <c r="G29" s="22" t="s">
+      <c r="G29" s="19" t="s">
         <v>92</v>
       </c>
       <c r="H29" s="21" t="s">
@@ -6705,7 +6695,7 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7"/>
-      <c r="B32" s="19"/>
+      <c r="B32" s="18"/>
       <c r="C32" s="14"/>
       <c r="D32" s="14"/>
       <c r="E32" s="14"/>
@@ -6724,7 +6714,7 @@
       <c r="A33" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="B33" s="18"/>
+      <c r="B33" s="17"/>
       <c r="C33" s="12"/>
       <c r="D33" s="12"/>
       <c r="E33" s="12"/>
@@ -6991,10 +6981,10 @@
         <v>49</v>
       </c>
       <c r="G38" s="3"/>
-      <c r="H38" s="17" t="s">
+      <c r="H38" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="I38" s="17" t="s">
+      <c r="I38" s="20" t="s">
         <v>58</v>
       </c>
       <c r="J38" s="6"/>
@@ -7014,8 +7004,8 @@
       <c r="E39" s="8"/>
       <c r="F39" s="8"/>
       <c r="G39" s="3"/>
-      <c r="H39" s="17"/>
-      <c r="I39" s="17"/>
+      <c r="H39" s="20"/>
+      <c r="I39" s="20"/>
       <c r="J39" s="6"/>
       <c r="K39" s="2"/>
       <c r="L39" s="2"/>
@@ -7024,7 +7014,7 @@
       <c r="O39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="19"/>
+      <c r="B40" s="18"/>
       <c r="C40" s="14"/>
       <c r="D40" s="14"/>
       <c r="E40" s="14"/>
@@ -7043,7 +7033,7 @@
       <c r="A41" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="B41" s="18"/>
+      <c r="B41" s="17"/>
       <c r="C41" s="12"/>
       <c r="D41" s="12"/>
       <c r="E41" s="12"/>
@@ -7251,8 +7241,8 @@
       <c r="O47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="19"/>
-      <c r="B48" s="19"/>
+      <c r="A48" s="18"/>
+      <c r="B48" s="18"/>
       <c r="C48" s="14"/>
       <c r="D48" s="14"/>
       <c r="E48" s="14"/>
@@ -7268,10 +7258,10 @@
       <c r="O48" s="15"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="18" t="s">
+      <c r="A49" s="17" t="s">
         <v>198</v>
       </c>
-      <c r="B49" s="18"/>
+      <c r="B49" s="17"/>
       <c r="C49" s="12"/>
       <c r="D49" s="12"/>
       <c r="E49" s="12"/>
@@ -7330,14 +7320,14 @@
       <c r="E52" s="4"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I52" s="3"/>
       <c r="J52" s="2" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="K52" s="2"/>
       <c r="L52" s="2"/>

</xml_diff>